<commit_message>
Set up Celery worker with Redis broker
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandi\Whatsapp-recruiting-agent\tests\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84416D89-3C66-4733-A344-E1AE4CC1FD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDCF67C0-4599-4A95-82A6-5139F348AB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6C9D8587-6826-4366-80CD-CC6319D470DB}"/>
+    <workbookView xWindow="4000" yWindow="1670" windowWidth="14400" windowHeight="8170" xr2:uid="{6C9D8587-6826-4366-80CD-CC6319D470DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>name</t>
   </si>
@@ -412,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43C3EF2D-3B0D-4020-808B-861F225314FE}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -462,6 +462,17 @@
         <v>8</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>5682919739</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Nanditha/queue worker setup (#27)
* Excel upload endpoint + parsing tests

* Add validation and deduplication logic with tests

* Add validation and deduplication logic with tests

* Task 3: Load Supabase credentials from environment variables, ignore .env

* Set up Celery worker with Redis broker

* Add celery to requirements.txt

* Add python-dotenv to requirements

* Update requirements.txt

* Update main.py

* retrigger CI

* retrigger CI

* Add status transition logic and tests
</commit_message>
<xml_diff>
--- a/tests/data/sample.xlsx
+++ b/tests/data/sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nandi\Whatsapp-recruiting-agent\tests\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84416D89-3C66-4733-A344-E1AE4CC1FD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDCF67C0-4599-4A95-82A6-5139F348AB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6C9D8587-6826-4366-80CD-CC6319D470DB}"/>
+    <workbookView xWindow="4000" yWindow="1670" windowWidth="14400" windowHeight="8170" xr2:uid="{6C9D8587-6826-4366-80CD-CC6319D470DB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>name</t>
   </si>
@@ -412,7 +412,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43C3EF2D-3B0D-4020-808B-861F225314FE}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -462,6 +462,17 @@
         <v>8</v>
       </c>
     </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>5682919739</v>
+      </c>
+      <c r="C5" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>